<commit_message>
Audit model; show n.m. for zero-denominator ratios
Add audit_model.py, which recalculates edited copies in LibreOffice and
compares every monthly and annual cell with a Python recalculation
across 12 scenario and edge-case runs, plus accounting identities and
breakeven tests. Fix ratios that returned 0 instead of n.m. when the
denominator was zero, make the dependent checks handle that, and add a
capacity-cap indicator.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018QDw9YR2j2g8LL97XVTLTN
</commit_message>
<xml_diff>
--- a/Joby_Financial_Model.xlsx
+++ b/Joby_Financial_Model.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="305">
   <si>
     <t xml:space="preserve">Joby Aviation - Air Taxi Route Financial Model (Prototype)</t>
   </si>
@@ -251,7 +251,13 @@
     <t xml:space="preserve">Annual rates</t>
   </si>
   <si>
-    <t xml:space="preserve">Rates are weighted by their natural base (e.g. load factor = passengers / seats; fare = revenue / passengers), never simple averages of months.</t>
+    <t xml:space="preserve">Rates are weighted by their natural base (e.g. load factor = passengers / seats; fare = revenue / passengers), never simple averages of months. Any ratio with a zero denominator (e.g. margin with no revenue, cost per flight with no flights) shows 'n.m.' (not meaningful) rather than 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load factor is capped at 100%. The Financial Model shows how many months demand growth exceeds seat capacity (information only).</t>
   </si>
   <si>
     <t xml:space="preserve">Recalculation</t>
@@ -797,10 +803,10 @@
     <t xml:space="preserve">Revenue, total variable costs, route operating profit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Revenue reconciles to passengers x weighted average fare</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual.</t>
+    <t xml:space="preserve">Revenue reconciles to passengers x average fare, month by month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual revenue = sum of (monthly passengers x monthly fare).</t>
   </si>
   <si>
     <t xml:space="preserve">Variable costs reconcile (flight + passenger = total)</t>
@@ -818,6 +824,9 @@
     <t xml:space="preserve">Contribution per flight x completed flights = contribution profit</t>
   </si>
   <si>
+    <t xml:space="preserve">Annual (zero flights must mean zero contribution).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cumulative route operating profit = annual total</t>
   </si>
   <si>
@@ -837,6 +846,12 @@
   </si>
   <si>
     <t xml:space="preserve">OVERALL MODEL STATUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months where demand exceeds seat capacity (load factor capped at 100%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information only. Above zero means the demand growth assumption implies more passengers than seats; the excess is not flown or counted as revenue.</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario Comparison - Base / Upside / Downside</t>
@@ -1101,7 +1116,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFF2F7FC"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -1186,7 +1201,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1451,6 +1466,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1488,7 +1507,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -1508,6 +1527,13 @@
         <b val="1"/>
         <color rgb="FFC00000"/>
       </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <colors>
@@ -1547,7 +1573,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFF2F7FC"/>
       <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1754,7 +1780,7 @@
     <tabColor rgb="FF2F5597"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -2066,7 +2092,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
         <v>65</v>
       </c>
@@ -2082,21 +2108,21 @@
         <v>68</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9" t="s">
+    <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="B48" s="10"/>
-      <c r="C48" s="10"/>
-      <c r="D48" s="10"/>
-    </row>
-    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="11" t="s">
+      <c r="B47" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B49" s="12" t="s">
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
         <v>71</v>
       </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
@@ -2112,6 +2138,14 @@
       </c>
       <c r="B51" s="12" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B52" s="12" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -2151,7 +2185,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2162,7 +2196,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2178,73 +2212,73 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G4" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C6" s="17" t="n">
         <f aca="false">MATCH($C$5,$C$9:$E$9,0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C7" s="6" t="str">
         <f aca="false">'Financial Model'!$C$70</f>
         <v>ALL 19 CHECKS PASS</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -2255,13 +2289,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D11" s="20"/>
       <c r="E11" s="20"/>
@@ -2270,18 +2304,18 @@
         <v>Route A: Downtown - Airport</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D12" s="20"/>
       <c r="E12" s="20"/>
@@ -2290,108 +2324,108 @@
         <v>Piloted eVTOL air taxi</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>46388</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F13" s="25" t="n">
         <f aca="false">$C13</f>
         <v>46388</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>4</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F14" s="27" t="n">
         <f aca="false">$C14</f>
         <v>4</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>32</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F15" s="27" t="n">
         <f aca="false">$C15</f>
         <v>32</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C16" s="26" t="n">
         <v>28</v>
       </c>
       <c r="D16" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F16" s="27" t="n">
         <f aca="false">$C16</f>
         <v>28</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
@@ -2402,10 +2436,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C19" s="28" t="n">
         <v>0.95</v>
@@ -2421,15 +2455,15 @@
         <v>0.95</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C20" s="30" t="n">
         <v>175</v>
@@ -2445,15 +2479,15 @@
         <v>175</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C21" s="28" t="n">
         <v>0.6</v>
@@ -2469,15 +2503,15 @@
         <v>0.6</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C22" s="30" t="n">
         <v>300</v>
@@ -2493,15 +2527,15 @@
         <v>300</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C23" s="30" t="n">
         <v>12</v>
@@ -2517,15 +2551,15 @@
         <v>12</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C24" s="32" t="n">
         <v>90000</v>
@@ -2541,12 +2575,12 @@
         <v>90000</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
@@ -2557,10 +2591,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C27" s="34" t="n">
         <v>0</v>
@@ -2576,15 +2610,15 @@
         <v>0</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B28" s="16" t="s">
         <v>136</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>134</v>
       </c>
       <c r="C28" s="34" t="n">
         <v>0.015</v>
@@ -2600,15 +2634,15 @@
         <v>0.015</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C29" s="34" t="n">
         <v>0</v>
@@ -2624,12 +2658,12 @@
         <v>0</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -2640,10 +2674,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B32" s="36" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C32" s="36"/>
       <c r="D32" s="36"/>
@@ -2653,10 +2687,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B33" s="36" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C33" s="36"/>
       <c r="D33" s="36"/>
@@ -2666,10 +2700,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B34" s="36" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C34" s="36"/>
       <c r="D34" s="36"/>
@@ -2679,7 +2713,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B36" s="10"/>
       <c r="C36" s="10"/>
@@ -2690,7 +2724,7 @@
     </row>
     <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="36" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B37" s="36"/>
       <c r="C37" s="36"/>
@@ -2701,7 +2735,7 @@
     </row>
     <row r="38" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="36" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B38" s="36"/>
       <c r="C38" s="36"/>
@@ -2712,7 +2746,7 @@
     </row>
     <row r="39" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="36" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B39" s="36"/>
       <c r="C39" s="36"/>
@@ -2723,7 +2757,7 @@
     </row>
     <row r="40" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="36" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B40" s="36"/>
       <c r="C40" s="36"/>
@@ -2734,7 +2768,7 @@
     </row>
     <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="36" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B41" s="36"/>
       <c r="C41" s="36"/>
@@ -2790,7 +2824,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -2802,7 +2836,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2822,7 +2856,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2853,60 +2887,60 @@
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E6" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J6" s="19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L6" s="19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N6" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O6" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P6" s="19" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C7" s="39" t="n">
         <v>1</v>
@@ -2960,10 +2994,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="37" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C8" s="40" t="n">
         <f aca="false">EDATE(Assumptions!$F$13,C$7-1)</f>
@@ -3018,7 +3052,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -3038,10 +3072,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C11" s="41" t="n">
         <f aca="false">Assumptions!$F$16</f>
@@ -3096,15 +3130,15 @@
         <v>336</v>
       </c>
       <c r="P11" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C12" s="41" t="n">
         <f aca="false">Assumptions!$F$15</f>
@@ -3155,19 +3189,19 @@
         <v>32</v>
       </c>
       <c r="O12" s="44" t="n">
-        <f aca="false">IF(O11=0,0,O22/O11)</f>
+        <f aca="false">IF(O11=0,"n.m.",O22/O11)</f>
         <v>32</v>
       </c>
       <c r="P12" s="43" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C13" s="45" t="n">
         <f aca="false">(1+Assumptions!$F$27)^(C$7-1)</f>
@@ -3222,10 +3256,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C14" s="45" t="n">
         <f aca="false">(1+Assumptions!$F$28)^(C$7-1)</f>
@@ -3280,10 +3314,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="C15" s="45" t="n">
         <f aca="false">(1+Assumptions!$F$29)^(C$7-1)</f>
@@ -3338,10 +3372,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C16" s="47" t="n">
         <f aca="false">Assumptions!$F$19</f>
@@ -3392,19 +3426,19 @@
         <v>0.95</v>
       </c>
       <c r="O16" s="29" t="n">
-        <f aca="false">IF(O22=0,0,O23/O22)</f>
+        <f aca="false">IF(O22=0,"n.m.",O23/O22)</f>
         <v>0.95</v>
       </c>
       <c r="P16" s="43" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C17" s="48" t="n">
         <f aca="false">MIN(1,MAX(0,Assumptions!$F$21*C14))</f>
@@ -3455,19 +3489,19 @@
         <v>0.706769362440316</v>
       </c>
       <c r="O17" s="29" t="n">
-        <f aca="false">IF(O24=0,0,O25/O24)</f>
+        <f aca="false">IF(O24=0,"n.m.",O25/O24)</f>
         <v>0.65206057153845</v>
       </c>
       <c r="P17" s="43" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C18" s="49" t="n">
         <f aca="false">Assumptions!$F$22*C15</f>
@@ -3518,19 +3552,19 @@
         <v>300</v>
       </c>
       <c r="O18" s="31" t="n">
-        <f aca="false">IF(O23=0,0,O30/O23)</f>
+        <f aca="false">IF(O23=0,"n.m.",O30/O23)</f>
         <v>300</v>
       </c>
       <c r="P18" s="43" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C19" s="49" t="n">
         <f aca="false">Assumptions!$F$23*C15</f>
@@ -3581,16 +3615,16 @@
         <v>12</v>
       </c>
       <c r="O19" s="31" t="n">
-        <f aca="false">IF(O25=0,0,O31/O25)</f>
+        <f aca="false">IF(O25=0,"n.m.",O31/O25)</f>
         <v>12</v>
       </c>
       <c r="P19" s="43" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="10"/>
@@ -3613,7 +3647,7 @@
         <v>45</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C22" s="50" t="n">
         <f aca="false">C11*C12</f>
@@ -3668,7 +3702,7 @@
         <v>10752</v>
       </c>
       <c r="P22" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3676,7 +3710,7 @@
         <v>47</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C23" s="50" t="n">
         <f aca="false">C22*C16</f>
@@ -3731,15 +3765,15 @@
         <v>10214.4</v>
       </c>
       <c r="P23" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C24" s="50" t="n">
         <f aca="false">C23*Assumptions!$F$14</f>
@@ -3794,7 +3828,7 @@
         <v>40857.6</v>
       </c>
       <c r="P24" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3802,7 +3836,7 @@
         <v>51</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C25" s="51" t="n">
         <f aca="false">C24*C17</f>
@@ -3857,12 +3891,12 @@
         <v>26641.6300076894</v>
       </c>
       <c r="P25" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>
@@ -3882,10 +3916,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">Assumptions!$F$20*C13</f>
@@ -3936,11 +3970,11 @@
         <v>175</v>
       </c>
       <c r="O28" s="31" t="n">
-        <f aca="false">IF(O25=0,0,O29/O25)</f>
+        <f aca="false">IF(O25=0,"n.m.",O29/O25)</f>
         <v>175</v>
       </c>
       <c r="P28" s="43" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3948,7 +3982,7 @@
         <v>53</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C29" s="52" t="n">
         <f aca="false">C25*C28</f>
@@ -4003,15 +4037,15 @@
         <v>4662285.25134564</v>
       </c>
       <c r="P29" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C30" s="53" t="n">
         <f aca="false">C23*C18</f>
@@ -4066,7 +4100,7 @@
         <v>3064320</v>
       </c>
       <c r="P30" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4074,7 +4108,7 @@
         <v>57</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C31" s="53" t="n">
         <f aca="false">C25*C19</f>
@@ -4129,15 +4163,15 @@
         <v>319699.560092273</v>
       </c>
       <c r="P31" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B32" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="C32" s="54" t="n">
         <f aca="false">C30+C31</f>
@@ -4192,15 +4226,15 @@
         <v>3384019.56009227</v>
       </c>
       <c r="P32" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C33" s="52" t="n">
         <f aca="false">C29-C32</f>
@@ -4255,141 +4289,141 @@
         <v>1278265.69125337</v>
       </c>
       <c r="P33" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="16" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C34" s="48" t="n">
-        <f aca="false">IF(C29=0,0,C33/C29)</f>
+        <f aca="false">IF(C29=0,"n.m.",C33/C29)</f>
         <v>0.217142857142857</v>
       </c>
       <c r="D34" s="48" t="n">
-        <f aca="false">IF(D29=0,0,D33/D29)</f>
+        <f aca="false">IF(D29=0,"n.m.",D33/D29)</f>
         <v>0.227698803659395</v>
       </c>
       <c r="E34" s="48" t="n">
-        <f aca="false">IF(E29=0,0,E33/E29)</f>
+        <f aca="false">IF(E29=0,"n.m.",E33/E29)</f>
         <v>0.238098750966328</v>
       </c>
       <c r="F34" s="48" t="n">
-        <f aca="false">IF(F29=0,0,F33/F29)</f>
+        <f aca="false">IF(F29=0,"n.m.",F33/F29)</f>
         <v>0.248345004470696</v>
       </c>
       <c r="G34" s="48" t="n">
-        <f aca="false">IF(G29=0,0,G33/G29)</f>
+        <f aca="false">IF(G29=0,"n.m.",G33/G29)</f>
         <v>0.258439835509483</v>
       </c>
       <c r="H34" s="48" t="n">
-        <f aca="false">IF(H29=0,0,H33/H29)</f>
+        <f aca="false">IF(H29=0,"n.m.",H33/H29)</f>
         <v>0.268385481853114</v>
       </c>
       <c r="I34" s="48" t="n">
-        <f aca="false">IF(I29=0,0,I33/I29)</f>
+        <f aca="false">IF(I29=0,"n.m.",I33/I29)</f>
         <v>0.27818414820152</v>
       </c>
       <c r="J34" s="48" t="n">
-        <f aca="false">IF(J29=0,0,J33/J29)</f>
+        <f aca="false">IF(J29=0,"n.m.",J33/J29)</f>
         <v>0.287838006672856</v>
       </c>
       <c r="K34" s="48" t="n">
-        <f aca="false">IF(K29=0,0,K33/K29)</f>
+        <f aca="false">IF(K29=0,"n.m.",K33/K29)</f>
         <v>0.297349197285009</v>
       </c>
       <c r="L34" s="48" t="n">
-        <f aca="false">IF(L29=0,0,L33/L29)</f>
+        <f aca="false">IF(L29=0,"n.m.",L33/L29)</f>
         <v>0.306719828429988</v>
       </c>
       <c r="M34" s="48" t="n">
-        <f aca="false">IF(M29=0,0,M33/M29)</f>
+        <f aca="false">IF(M29=0,"n.m.",M33/M29)</f>
         <v>0.315951977341297</v>
       </c>
       <c r="N34" s="48" t="n">
-        <f aca="false">IF(N29=0,0,N33/N29)</f>
+        <f aca="false">IF(N29=0,"n.m.",N33/N29)</f>
         <v>0.325047690554409</v>
       </c>
       <c r="O34" s="29" t="n">
-        <f aca="false">IF(O29=0,0,O33/O29)</f>
+        <f aca="false">IF(O29=0,"n.m.",O33/O29)</f>
         <v>0.27417148937518</v>
       </c>
       <c r="P34" s="43" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="16" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C35" s="49" t="n">
-        <f aca="false">IF(C23=0,0,C33/C23)</f>
+        <f aca="false">IF(C23=0,"n.m.",C33/C23)</f>
         <v>91.2</v>
       </c>
       <c r="D35" s="49" t="n">
-        <f aca="false">IF(D23=0,0,D33/D23)</f>
+        <f aca="false">IF(D23=0,"n.m.",D33/D23)</f>
         <v>97.068</v>
       </c>
       <c r="E35" s="49" t="n">
-        <f aca="false">IF(E23=0,0,E33/E23)</f>
+        <f aca="false">IF(E23=0,"n.m.",E33/E23)</f>
         <v>103.02402</v>
       </c>
       <c r="F35" s="49" t="n">
-        <f aca="false">IF(F23=0,0,F33/F23)</f>
+        <f aca="false">IF(F23=0,"n.m.",F33/F23)</f>
         <v>109.0693803</v>
       </c>
       <c r="G35" s="49" t="n">
-        <f aca="false">IF(G23=0,0,G33/G23)</f>
+        <f aca="false">IF(G23=0,"n.m.",G33/G23)</f>
         <v>115.2054210045</v>
       </c>
       <c r="H35" s="49" t="n">
-        <f aca="false">IF(H23=0,0,H33/H23)</f>
+        <f aca="false">IF(H23=0,"n.m.",H33/H23)</f>
         <v>121.433502319567</v>
       </c>
       <c r="I35" s="49" t="n">
-        <f aca="false">IF(I23=0,0,I33/I23)</f>
+        <f aca="false">IF(I23=0,"n.m.",I33/I23)</f>
         <v>127.755004854361</v>
       </c>
       <c r="J35" s="49" t="n">
-        <f aca="false">IF(J23=0,0,J33/J23)</f>
+        <f aca="false">IF(J23=0,"n.m.",J33/J23)</f>
         <v>134.171329927176</v>
       </c>
       <c r="K35" s="49" t="n">
-        <f aca="false">IF(K23=0,0,K33/K23)</f>
+        <f aca="false">IF(K23=0,"n.m.",K33/K23)</f>
         <v>140.683899876084</v>
       </c>
       <c r="L35" s="49" t="n">
-        <f aca="false">IF(L23=0,0,L33/L23)</f>
+        <f aca="false">IF(L23=0,"n.m.",L33/L23)</f>
         <v>147.294158374225</v>
       </c>
       <c r="M35" s="49" t="n">
-        <f aca="false">IF(M23=0,0,M33/M23)</f>
+        <f aca="false">IF(M23=0,"n.m.",M33/M23)</f>
         <v>154.003570749838</v>
       </c>
       <c r="N35" s="49" t="n">
-        <f aca="false">IF(N23=0,0,N33/N23)</f>
+        <f aca="false">IF(N23=0,"n.m.",N33/N23)</f>
         <v>160.813624311086</v>
       </c>
       <c r="O35" s="31" t="n">
-        <f aca="false">IF(O23=0,0,O33/O23)</f>
+        <f aca="false">IF(O23=0,"n.m.",O33/O23)</f>
         <v>125.14349264307</v>
       </c>
       <c r="P35" s="43" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C36" s="53" t="n">
         <f aca="false">Assumptions!$F$24*C15</f>
@@ -4444,15 +4478,15 @@
         <v>1080000</v>
       </c>
       <c r="P36" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C37" s="56" t="n">
         <f aca="false">C33-C36</f>
@@ -4507,78 +4541,78 @@
         <v>198265.691253371</v>
       </c>
       <c r="P37" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="16" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C38" s="48" t="n">
-        <f aca="false">IF(C29=0,0,C37/C29)</f>
+        <f aca="false">IF(C29=0,"n.m.",C37/C29)</f>
         <v>-0.0346025778732546</v>
       </c>
       <c r="D38" s="48" t="n">
-        <f aca="false">IF(D29=0,0,D37/D29)</f>
+        <f aca="false">IF(D29=0,"n.m.",D37/D29)</f>
         <v>-0.0203262554697793</v>
       </c>
       <c r="E38" s="48" t="n">
-        <f aca="false">IF(E29=0,0,E37/E29)</f>
+        <f aca="false">IF(E29=0,"n.m.",E37/E29)</f>
         <v>-0.00626091320034579</v>
       </c>
       <c r="F38" s="48" t="n">
-        <f aca="false">IF(F29=0,0,F37/F29)</f>
+        <f aca="false">IF(F29=0,"n.m.",F37/F29)</f>
         <v>0.00759656686806172</v>
       </c>
       <c r="G38" s="48" t="n">
-        <f aca="false">IF(G29=0,0,G37/G29)</f>
+        <f aca="false">IF(G29=0,"n.m.",G37/G29)</f>
         <v>0.021249256590631</v>
       </c>
       <c r="H38" s="48" t="n">
-        <f aca="false">IF(H29=0,0,H37/H29)</f>
+        <f aca="false">IF(H29=0,"n.m.",H37/H29)</f>
         <v>0.0347001824256742</v>
       </c>
       <c r="I38" s="48" t="n">
-        <f aca="false">IF(I29=0,0,I37/I29)</f>
+        <f aca="false">IF(I29=0,"n.m.",I37/I29)</f>
         <v>0.0479523261055198</v>
       </c>
       <c r="J38" s="48" t="n">
-        <f aca="false">IF(J29=0,0,J37/J29)</f>
+        <f aca="false">IF(J29=0,"n.m.",J37/J29)</f>
         <v>0.0610086252974862</v>
       </c>
       <c r="K38" s="48" t="n">
-        <f aca="false">IF(K29=0,0,K37/K29)</f>
+        <f aca="false">IF(K29=0,"n.m.",K37/K29)</f>
         <v>0.0738719742550883</v>
       </c>
       <c r="L38" s="48" t="n">
-        <f aca="false">IF(L29=0,0,L37/L29)</f>
+        <f aca="false">IF(L29=0,"n.m.",L37/L29)</f>
         <v>0.0865452244596225</v>
       </c>
       <c r="M38" s="48" t="n">
-        <f aca="false">IF(M29=0,0,M37/M29)</f>
+        <f aca="false">IF(M29=0,"n.m.",M37/M29)</f>
         <v>0.0990311852522669</v>
       </c>
       <c r="N38" s="48" t="n">
-        <f aca="false">IF(N29=0,0,N37/N29)</f>
+        <f aca="false">IF(N29=0,"n.m.",N37/N29)</f>
         <v>0.111332624456843</v>
       </c>
       <c r="O38" s="29" t="n">
-        <f aca="false">IF(O29=0,0,O37/O29)</f>
+        <f aca="false">IF(O29=0,"n.m.",O37/O29)</f>
         <v>0.0425254313206484</v>
       </c>
       <c r="P38" s="43" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C39" s="53" t="n">
         <f aca="false">C37</f>
@@ -4633,12 +4667,12 @@
         <v>198265.691253371</v>
       </c>
       <c r="P39" s="43" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
@@ -4658,10 +4692,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">C28-C19</f>
@@ -4712,19 +4746,19 @@
         <v>163</v>
       </c>
       <c r="O42" s="31" t="n">
-        <f aca="false">IF(O25=0,0,(O29-O31)/O25)</f>
+        <f aca="false">IF(O25=0,"n.m.",(O29-O31)/O25)</f>
         <v>163</v>
       </c>
       <c r="P42" s="43" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="16" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C43" s="53" t="n">
         <f aca="false">C24*C42</f>
@@ -4779,15 +4813,15 @@
         <v>6659788.8</v>
       </c>
       <c r="P43" s="43" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C44" s="48" t="n">
         <f aca="false">IF(C43&gt;0,(C30)/C43,"n.m.")</f>
@@ -4842,15 +4876,15 @@
         <v>0.460122699386503</v>
       </c>
       <c r="P44" s="43" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C45" s="58" t="n">
         <f aca="false">IF(C43&gt;0,(C30+C36)/C43,"n.m.")</f>
@@ -4905,15 +4939,15 @@
         <v>0.622290004151483</v>
       </c>
       <c r="P45" s="43" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C46" s="48" t="n">
         <f aca="false">IF(ISNUMBER(C45),C17-C45,"n.m.")</f>
@@ -4968,12 +5002,12 @@
         <v>0.0297705673869674</v>
       </c>
       <c r="P46" s="43" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="59" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B47" s="59"/>
       <c r="C47" s="59"/>
@@ -4993,7 +5027,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B49" s="10"/>
       <c r="C49" s="10"/>
@@ -5013,14 +5047,14 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="60" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B50" s="61"/>
       <c r="C50" s="60" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D50" s="60" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E50" s="61"/>
       <c r="F50" s="61"/>
@@ -5037,235 +5071,235 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="16" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C51" s="62" t="str">
         <f aca="false">IF(ISNUMBER(Assumptions!$C$6),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D51" s="43" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C52" s="62" t="str">
         <f aca="false">IF(AND(MIN(Assumptions!$C$21:$E$21)&gt;=0,MAX(Assumptions!$C$21:$E$21)&lt;=1),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D52" s="43" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="16" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C53" s="62" t="str">
         <f aca="false">IF(AND(MIN(Assumptions!$C$19:$E$19)&gt;=0,MAX(Assumptions!$C$19:$E$19)&lt;=1),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D53" s="43" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C54" s="62" t="str">
         <f aca="false">IF(AND(MIN($C$17:$N$17)&gt;=0,MAX($C$17:$N$17)&lt;=1),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D54" s="43" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="16" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C55" s="62" t="str">
         <f aca="false">IF(AND(MIN($C$16:$N$16)&gt;=0,MAX($C$16:$N$16)&lt;=1),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D55" s="43" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="16" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C56" s="62" t="str">
         <f aca="false">IF(AND(Assumptions!$C$14&gt;=0,Assumptions!$C$15&gt;=0,Assumptions!$C$16&gt;=0),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D56" s="43" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="16" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C57" s="62" t="str">
         <f aca="false">IF(AND(MIN($C$22:$N$22)&gt;=0,MIN($C$23:$N$23)&gt;=0,SUMPRODUCT(($C$23:$N$23&gt;$C$22:$N$22)*1)=0),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D57" s="43" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="16" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C58" s="62" t="str">
         <f aca="false">IF(SUMPRODUCT(($C$25:$N$25&gt;$C$24:$N$24+0.000001)*1)=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D58" s="43" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="16" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C59" s="62" t="str">
         <f aca="false">IF(MIN(Assumptions!$C$22:$E$24)&gt;=0,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D59" s="43" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="16" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C60" s="62" t="str">
         <f aca="false">IF(AND(MIN($C$30:$N$30)&gt;=0,MIN($C$31:$N$31)&gt;=0,MIN($C$36:$N$36)&gt;=0),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D60" s="43" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="16" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C61" s="62" t="str">
         <f aca="false">IF(AND(ABS($O$29-SUM($C$29:$N$29))&lt;0.01,ABS($O$32-SUM($C$32:$N$32))&lt;0.01,ABS($O$37-SUM($C$37:$N$37))&lt;0.01),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D61" s="43" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C62" s="62" t="str">
-        <f aca="false">IF(ABS($O$29-$O$25*$O$28)&lt;0.01,"PASS","FAIL")</f>
+        <f aca="false">IF(ABS($O$29-SUMPRODUCT($C$25:$N$25,$C$28:$N$28))&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D62" s="43" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C63" s="62" t="str">
         <f aca="false">IF(ABS($O$30+$O$31-$O$32)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D63" s="43" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="16" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C64" s="62" t="str">
         <f aca="false">IF(ABS($O$29-$O$30-$O$31-$O$36-$O$37)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D64" s="43" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C65" s="62" t="str">
-        <f aca="false">IF(ABS($O$35*$O$23-$O$33)&lt;0.01,"PASS","FAIL")</f>
+        <f aca="false">IF(IF(ISNUMBER($O$35),ABS($O$35*$O$23-$O$33)&lt;0.01,ABS($O$33)&lt;0.01),"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D65" s="43" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="16" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C66" s="62" t="str">
         <f aca="false">IF(ABS($O$39-$O$37)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D66" s="43" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="16" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C67" s="62" t="str">
         <f aca="false">IF(ABS(INDEX('Scenario Comparison'!$C$23:$E$23,Assumptions!$C$6)-$O$29)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D67" s="43" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="16" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C68" s="62" t="str">
         <f aca="false">IF(ABS(INDEX('Scenario Comparison'!$C$29:$E$29,Assumptions!$C$6)-$O$37)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D68" s="43" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="16" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C69" s="62" t="str">
         <f aca="false">IF(ABS(INDEX('Scenario Comparison'!$C$20:$E$20,Assumptions!$C$6)-$O$25)&lt;0.01,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="D69" s="43" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="63" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B70" s="64"/>
       <c r="C70" s="65" t="str">
@@ -5275,6 +5309,18 @@
       <c r="D70" s="65"/>
       <c r="E70" s="65"/>
       <c r="F70" s="65"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="C72" s="66" t="n">
+        <f aca="false">SUMPRODUCT((Assumptions!$F$21*$C$14:$N$14&gt;1)*1)</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="43" t="s">
+        <v>266</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5312,6 +5358,11 @@
       <formula>LEFT($C$70,3)&lt;&gt;"ALL"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C72">
+    <cfRule type="cellIs" priority="9" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5341,7 +5392,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5361,7 +5412,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5386,28 +5437,28 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E5" s="19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
@@ -5420,7 +5471,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -5440,10 +5491,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C7" s="47" t="n">
         <f aca="false">Assumptions!$C$19</f>
@@ -5468,20 +5519,20 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="C8" s="66" t="n">
+        <v>121</v>
+      </c>
+      <c r="C8" s="67" t="n">
         <f aca="false">Assumptions!$C$20</f>
         <v>175</v>
       </c>
-      <c r="D8" s="66" t="n">
+      <c r="D8" s="67" t="n">
         <f aca="false">Assumptions!$D$20</f>
         <v>190</v>
       </c>
-      <c r="E8" s="66" t="n">
+      <c r="E8" s="67" t="n">
         <f aca="false">Assumptions!$E$20</f>
         <v>160</v>
       </c>
@@ -5496,10 +5547,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C9" s="47" t="n">
         <f aca="false">Assumptions!$C$21</f>
@@ -5524,20 +5575,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="C10" s="66" t="n">
+        <v>186</v>
+      </c>
+      <c r="C10" s="67" t="n">
         <f aca="false">Assumptions!$C$22</f>
         <v>300</v>
       </c>
-      <c r="D10" s="66" t="n">
+      <c r="D10" s="67" t="n">
         <f aca="false">Assumptions!$D$22</f>
         <v>280</v>
       </c>
-      <c r="E10" s="66" t="n">
+      <c r="E10" s="67" t="n">
         <f aca="false">Assumptions!$E$22</f>
         <v>320</v>
       </c>
@@ -5552,20 +5603,20 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="66" t="n">
+        <v>121</v>
+      </c>
+      <c r="C11" s="67" t="n">
         <f aca="false">Assumptions!$C$23</f>
         <v>12</v>
       </c>
-      <c r="D11" s="66" t="n">
+      <c r="D11" s="67" t="n">
         <f aca="false">Assumptions!$D$23</f>
         <v>10</v>
       </c>
-      <c r="E11" s="66" t="n">
+      <c r="E11" s="67" t="n">
         <f aca="false">Assumptions!$E$23</f>
         <v>15</v>
       </c>
@@ -5580,20 +5631,20 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="C12" s="67" t="n">
+        <v>132</v>
+      </c>
+      <c r="C12" s="68" t="n">
         <f aca="false">Assumptions!$C$24</f>
         <v>90000</v>
       </c>
-      <c r="D12" s="67" t="n">
+      <c r="D12" s="68" t="n">
         <f aca="false">Assumptions!$D$24</f>
         <v>85000</v>
       </c>
-      <c r="E12" s="67" t="n">
+      <c r="E12" s="68" t="n">
         <f aca="false">Assumptions!$E$24</f>
         <v>100000</v>
       </c>
@@ -5608,91 +5659,91 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="C13" s="68" t="n">
+        <v>280</v>
+      </c>
+      <c r="C13" s="69" t="n">
         <f aca="false">Assumptions!$C$27</f>
         <v>0</v>
       </c>
-      <c r="D13" s="68" t="n">
+      <c r="D13" s="69" t="n">
         <f aca="false">Assumptions!$D$27</f>
         <v>0.0025</v>
       </c>
-      <c r="E13" s="68" t="n">
+      <c r="E13" s="69" t="n">
         <f aca="false">Assumptions!$E$27</f>
         <v>-0.005</v>
       </c>
-      <c r="F13" s="69" t="n">
+      <c r="F13" s="70" t="n">
         <f aca="false">D13-C13</f>
         <v>0.0025</v>
       </c>
-      <c r="G13" s="69" t="n">
+      <c r="G13" s="70" t="n">
         <f aca="false">E13-C13</f>
         <v>-0.005</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="C14" s="68" t="n">
+        <v>280</v>
+      </c>
+      <c r="C14" s="69" t="n">
         <f aca="false">Assumptions!$C$28</f>
         <v>0.015</v>
       </c>
-      <c r="D14" s="68" t="n">
+      <c r="D14" s="69" t="n">
         <f aca="false">Assumptions!$D$28</f>
         <v>0.02</v>
       </c>
-      <c r="E14" s="68" t="n">
+      <c r="E14" s="69" t="n">
         <f aca="false">Assumptions!$E$28</f>
         <v>0.005</v>
       </c>
-      <c r="F14" s="69" t="n">
+      <c r="F14" s="70" t="n">
         <f aca="false">D14-C14</f>
         <v>0.005</v>
       </c>
-      <c r="G14" s="69" t="n">
+      <c r="G14" s="70" t="n">
         <f aca="false">E14-C14</f>
         <v>-0.01</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="C15" s="68" t="n">
+        <v>280</v>
+      </c>
+      <c r="C15" s="69" t="n">
         <f aca="false">Assumptions!$C$29</f>
         <v>0</v>
       </c>
-      <c r="D15" s="68" t="n">
+      <c r="D15" s="69" t="n">
         <f aca="false">Assumptions!$D$29</f>
         <v>-0.0025</v>
       </c>
-      <c r="E15" s="68" t="n">
+      <c r="E15" s="69" t="n">
         <f aca="false">Assumptions!$E$29</f>
         <v>0.005</v>
       </c>
-      <c r="F15" s="69" t="n">
+      <c r="F15" s="70" t="n">
         <f aca="false">D15-C15</f>
         <v>-0.0025</v>
       </c>
-      <c r="G15" s="69" t="n">
+      <c r="G15" s="70" t="n">
         <f aca="false">E15-C15</f>
         <v>0.005</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -5715,7 +5766,7 @@
         <v>45</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C18" s="50" t="n">
         <f aca="false">O57</f>
@@ -5744,7 +5795,7 @@
         <v>47</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C19" s="50" t="n">
         <f aca="false">O58</f>
@@ -5773,7 +5824,7 @@
         <v>51</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C20" s="50" t="n">
         <f aca="false">O60</f>
@@ -5799,21 +5850,21 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C21" s="48" t="n">
-        <f aca="false">IF(O59=0,0,O60/O59)</f>
+        <f aca="false">IF(O59=0,"n.m.",O60/O59)</f>
         <v>0.65206057153845</v>
       </c>
       <c r="D21" s="48" t="n">
-        <f aca="false">IF(O77=0,0,O78/O77)</f>
+        <f aca="false">IF(O77=0,"n.m.",O78/O77)</f>
         <v>0.760018417927212</v>
       </c>
       <c r="E21" s="48" t="n">
-        <f aca="false">IF(O95=0,0,O96/O95)</f>
+        <f aca="false">IF(O95=0,"n.m.",O96/O95)</f>
         <v>0.534541036158996</v>
       </c>
       <c r="F21" s="48" t="n">
@@ -5825,26 +5876,26 @@
         <v>-0.117519535379454</v>
       </c>
       <c r="H21" s="43" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C22" s="49" t="n">
-        <f aca="false">IF(O60=0,0,O61/O60)</f>
+        <f aca="false">IF(O60=0,"n.m.",O61/O60)</f>
         <v>175</v>
       </c>
       <c r="D22" s="49" t="n">
-        <f aca="false">IF(O78=0,0,O79/O78)</f>
+        <f aca="false">IF(O78=0,"n.m.",O79/O78)</f>
         <v>192.747801204525</v>
       </c>
       <c r="E22" s="49" t="n">
-        <f aca="false">IF(O96=0,0,O97/O96)</f>
+        <f aca="false">IF(O96=0,"n.m.",O97/O96)</f>
         <v>155.626145283513</v>
       </c>
       <c r="F22" s="49" t="n">
@@ -5856,15 +5907,15 @@
         <v>-19.3738547164867</v>
       </c>
       <c r="H22" s="43" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C23" s="52" t="n">
         <f aca="false">O61</f>
@@ -5890,10 +5941,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="C24" s="53" t="n">
         <f aca="false">O64</f>
@@ -5916,7 +5967,7 @@
         <v>118279.73668579</v>
       </c>
       <c r="H24" s="43" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5924,7 +5975,7 @@
         <v>59</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C25" s="52" t="n">
         <f aca="false">O65</f>
@@ -5947,26 +5998,26 @@
         <v>-1560568.72150065</v>
       </c>
       <c r="H25" s="43" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C26" s="48" t="n">
-        <f aca="false">IF(O61=0,0,O65/O61)</f>
+        <f aca="false">IF(O61=0,"n.m.",O65/O61)</f>
         <v>0.27417148937518</v>
       </c>
       <c r="D26" s="48" t="n">
-        <f aca="false">IF(O79=0,0,O83/O79)</f>
+        <f aca="false">IF(O79=0,"n.m.",O83/O79)</f>
         <v>0.47753008087474</v>
       </c>
       <c r="E26" s="48" t="n">
-        <f aca="false">IF(O97=0,0,O101/O97)</f>
+        <f aca="false">IF(O97=0,"n.m.",O101/O97)</f>
         <v>-0.0876718501762202</v>
       </c>
       <c r="F26" s="48" t="n">
@@ -5981,21 +6032,21 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="C27" s="70" t="n">
-        <f aca="false">IF(O58=0,0,O65/O58)</f>
+        <v>186</v>
+      </c>
+      <c r="C27" s="71" t="n">
+        <f aca="false">IF(O58=0,"n.m.",O65/O58)</f>
         <v>125.14349264307</v>
       </c>
-      <c r="D27" s="70" t="n">
-        <f aca="false">IF(O76=0,0,O83/O76)</f>
+      <c r="D27" s="71" t="n">
+        <f aca="false">IF(O76=0,"n.m.",O83/O76)</f>
         <v>279.817115172529</v>
       </c>
-      <c r="E27" s="70" t="n">
-        <f aca="false">IF(O94=0,0,O101/O94)</f>
+      <c r="E27" s="71" t="n">
+        <f aca="false">IF(O94=0,"n.m.",O101/O94)</f>
         <v>-29.1731802090852</v>
       </c>
       <c r="F27" s="49" t="n">
@@ -6010,10 +6061,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C28" s="53" t="n">
         <f aca="false">O66</f>
@@ -6039,10 +6090,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C29" s="52" t="n">
         <f aca="false">O67</f>
@@ -6065,26 +6116,26 @@
         <v>-1714124.95879064</v>
       </c>
       <c r="H29" s="43" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C30" s="48" t="n">
-        <f aca="false">IF(O61=0,0,O67/O61)</f>
+        <f aca="false">IF(O61=0,"n.m.",O67/O61)</f>
         <v>0.0425254313206484</v>
       </c>
       <c r="D30" s="48" t="n">
-        <f aca="false">IF(O79=0,0,O85/O79)</f>
+        <f aca="false">IF(O79=0,"n.m.",O85/O79)</f>
         <v>0.312902412084906</v>
       </c>
       <c r="E30" s="48" t="n">
-        <f aca="false">IF(O97=0,0,O103/O97)</f>
+        <f aca="false">IF(O97=0,"n.m.",O103/O97)</f>
         <v>-0.47076429351592</v>
       </c>
       <c r="F30" s="48" t="n">
@@ -6099,10 +6150,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C31" s="48" t="n">
         <f aca="false">IF(O68&gt;0,O62/O68,"n.m.")</f>
@@ -6125,15 +6176,15 @@
         <v>0.126225158941928</v>
       </c>
       <c r="H31" s="43" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C32" s="58" t="n">
         <f aca="false">IF(O68&gt;0,(O62+O66)/O68,"n.m.")</f>
@@ -6156,33 +6207,33 @@
         <v>0.191282191636812</v>
       </c>
       <c r="H32" s="43" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>292</v>
-      </c>
-      <c r="C33" s="71" t="n">
+        <v>297</v>
+      </c>
+      <c r="C33" s="72" t="n">
         <f aca="false">COUNTIF(C67:N67,"&gt;0")</f>
         <v>9</v>
       </c>
-      <c r="D33" s="71" t="n">
+      <c r="D33" s="72" t="n">
         <f aca="false">COUNTIF(C85:N85,"&gt;0")</f>
         <v>12</v>
       </c>
-      <c r="E33" s="71" t="n">
+      <c r="E33" s="72" t="n">
         <f aca="false">COUNTIF(C103:N103,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="F33" s="71" t="n">
+      <c r="F33" s="72" t="n">
         <f aca="false">IF(AND(ISNUMBER(D33),ISNUMBER(C33)),D33-C33,"n.m.")</f>
         <v>3</v>
       </c>
-      <c r="G33" s="71" t="n">
+      <c r="G33" s="72" t="n">
         <f aca="false">IF(AND(ISNUMBER(E33),ISNUMBER(C33)),E33-C33,"n.m.")</f>
         <v>-9</v>
       </c>
@@ -6190,7 +6241,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -6210,73 +6261,73 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B36" s="72" t="s">
-        <v>141</v>
-      </c>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72"/>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
-      <c r="G36" s="72"/>
-      <c r="H36" s="72"/>
-      <c r="I36" s="72"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="72"/>
-      <c r="L36" s="72"/>
-      <c r="M36" s="72"/>
-      <c r="N36" s="72"/>
-      <c r="O36" s="72"/>
-      <c r="P36" s="72"/>
+        <v>82</v>
+      </c>
+      <c r="B36" s="73" t="s">
+        <v>143</v>
+      </c>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="73"/>
+      <c r="M36" s="73"/>
+      <c r="N36" s="73"/>
+      <c r="O36" s="73"/>
+      <c r="P36" s="73"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B37" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="C37" s="72"/>
-      <c r="D37" s="72"/>
-      <c r="E37" s="72"/>
-      <c r="F37" s="72"/>
-      <c r="G37" s="72"/>
-      <c r="H37" s="72"/>
-      <c r="I37" s="72"/>
-      <c r="J37" s="72"/>
-      <c r="K37" s="72"/>
-      <c r="L37" s="72"/>
-      <c r="M37" s="72"/>
-      <c r="N37" s="72"/>
-      <c r="O37" s="72"/>
-      <c r="P37" s="72"/>
+        <v>91</v>
+      </c>
+      <c r="B37" s="73" t="s">
+        <v>144</v>
+      </c>
+      <c r="C37" s="73"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="73"/>
+      <c r="G37" s="73"/>
+      <c r="H37" s="73"/>
+      <c r="I37" s="73"/>
+      <c r="J37" s="73"/>
+      <c r="K37" s="73"/>
+      <c r="L37" s="73"/>
+      <c r="M37" s="73"/>
+      <c r="N37" s="73"/>
+      <c r="O37" s="73"/>
+      <c r="P37" s="73"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B38" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="C38" s="72"/>
-      <c r="D38" s="72"/>
-      <c r="E38" s="72"/>
-      <c r="F38" s="72"/>
-      <c r="G38" s="72"/>
-      <c r="H38" s="72"/>
-      <c r="I38" s="72"/>
-      <c r="J38" s="72"/>
-      <c r="K38" s="72"/>
-      <c r="L38" s="72"/>
-      <c r="M38" s="72"/>
-      <c r="N38" s="72"/>
-      <c r="O38" s="72"/>
-      <c r="P38" s="72"/>
+        <v>92</v>
+      </c>
+      <c r="B38" s="73" t="s">
+        <v>145</v>
+      </c>
+      <c r="C38" s="73"/>
+      <c r="D38" s="73"/>
+      <c r="E38" s="73"/>
+      <c r="F38" s="73"/>
+      <c r="G38" s="73"/>
+      <c r="H38" s="73"/>
+      <c r="I38" s="73"/>
+      <c r="J38" s="73"/>
+      <c r="K38" s="73"/>
+      <c r="L38" s="73"/>
+      <c r="M38" s="73"/>
+      <c r="N38" s="73"/>
+      <c r="O38" s="73"/>
+      <c r="P38" s="73"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="59" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B40" s="59"/>
       <c r="C40" s="59"/>
@@ -6296,7 +6347,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -6316,55 +6367,55 @@
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="18" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D52" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F52" s="19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G52" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H52" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I52" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J52" s="19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K52" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L52" s="19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M52" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N52" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O52" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P52" s="19"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C53" s="17" t="n">
         <v>1</v>
@@ -6416,10 +6467,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C54" s="49" t="n">
         <f aca="false">Assumptions!$C$20*(1+Assumptions!$C$27)^(C$53-1)</f>
@@ -6473,10 +6524,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C55" s="48" t="n">
         <f aca="false">MIN(1,MAX(0,Assumptions!$C$21*(1+Assumptions!$C$28)^(C$53-1)))</f>
@@ -6530,10 +6581,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B56" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="B56" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="C56" s="45" t="n">
         <f aca="false">(1+Assumptions!$C$29)^(C$53-1)</f>
@@ -6590,7 +6641,7 @@
         <v>45</v>
       </c>
       <c r="B57" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C57" s="50" t="n">
         <f aca="false">Assumptions!$F$16*Assumptions!$F$15</f>
@@ -6650,7 +6701,7 @@
         <v>47</v>
       </c>
       <c r="B58" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C58" s="50" t="n">
         <f aca="false">C57*Assumptions!$C$19</f>
@@ -6707,10 +6758,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C59" s="50" t="n">
         <f aca="false">C58*Assumptions!$F$14</f>
@@ -6770,7 +6821,7 @@
         <v>51</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C60" s="50" t="n">
         <f aca="false">C59*C55</f>
@@ -6830,7 +6881,7 @@
         <v>53</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C61" s="53" t="n">
         <f aca="false">C60*C54</f>
@@ -6887,10 +6938,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C62" s="53" t="n">
         <f aca="false">C58*Assumptions!$C$22*C56</f>
@@ -6950,7 +7001,7 @@
         <v>57</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C63" s="53" t="n">
         <f aca="false">C60*Assumptions!$C$23*C56</f>
@@ -7007,10 +7058,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B64" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="B64" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="C64" s="53" t="n">
         <f aca="false">C62+C63</f>
@@ -7070,7 +7121,7 @@
         <v>59</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C65" s="53" t="n">
         <f aca="false">C61-C64</f>
@@ -7127,10 +7178,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C66" s="53" t="n">
         <f aca="false">Assumptions!$C$24*C56</f>
@@ -7187,10 +7238,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C67" s="53" t="n">
         <f aca="false">C65-C66</f>
@@ -7247,10 +7298,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="16" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B68" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C68" s="53" t="n">
         <f aca="false">C59*(C54-Assumptions!$C$23*C56)</f>
@@ -7307,55 +7358,55 @@
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="18" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C70" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D70" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E70" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F70" s="19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G70" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H70" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I70" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J70" s="19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K70" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L70" s="19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M70" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N70" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O70" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P70" s="19"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C71" s="17" t="n">
         <v>1</v>
@@ -7407,10 +7458,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B72" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C72" s="49" t="n">
         <f aca="false">Assumptions!$D$20*(1+Assumptions!$D$27)^(C$71-1)</f>
@@ -7464,10 +7515,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C73" s="48" t="n">
         <f aca="false">MIN(1,MAX(0,Assumptions!$D$21*(1+Assumptions!$D$28)^(C$71-1)))</f>
@@ -7521,10 +7572,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B74" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="B74" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="C74" s="45" t="n">
         <f aca="false">(1+Assumptions!$D$29)^(C$71-1)</f>
@@ -7581,7 +7632,7 @@
         <v>45</v>
       </c>
       <c r="B75" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C75" s="50" t="n">
         <f aca="false">Assumptions!$F$16*Assumptions!$F$15</f>
@@ -7641,7 +7692,7 @@
         <v>47</v>
       </c>
       <c r="B76" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C76" s="50" t="n">
         <f aca="false">C75*Assumptions!$D$19</f>
@@ -7698,10 +7749,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C77" s="50" t="n">
         <f aca="false">C76*Assumptions!$F$14</f>
@@ -7761,7 +7812,7 @@
         <v>51</v>
       </c>
       <c r="B78" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C78" s="50" t="n">
         <f aca="false">C77*C73</f>
@@ -7821,7 +7872,7 @@
         <v>53</v>
       </c>
       <c r="B79" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C79" s="53" t="n">
         <f aca="false">C78*C72</f>
@@ -7878,10 +7929,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C80" s="53" t="n">
         <f aca="false">C76*Assumptions!$D$22*C74</f>
@@ -7941,7 +7992,7 @@
         <v>57</v>
       </c>
       <c r="B81" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C81" s="53" t="n">
         <f aca="false">C78*Assumptions!$D$23*C74</f>
@@ -7998,10 +8049,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B82" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="B82" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="C82" s="53" t="n">
         <f aca="false">C80+C81</f>
@@ -8061,7 +8112,7 @@
         <v>59</v>
       </c>
       <c r="B83" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C83" s="53" t="n">
         <f aca="false">C79-C82</f>
@@ -8118,10 +8169,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C84" s="53" t="n">
         <f aca="false">Assumptions!$D$24*C74</f>
@@ -8178,10 +8229,10 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B85" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C85" s="53" t="n">
         <f aca="false">C83-C84</f>
@@ -8238,10 +8289,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="16" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B86" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C86" s="53" t="n">
         <f aca="false">C77*(C72-Assumptions!$D$23*C74)</f>
@@ -8298,55 +8349,55 @@
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C88" s="19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D88" s="19" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E88" s="19" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F88" s="19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G88" s="19" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H88" s="19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I88" s="19" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="J88" s="19" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="K88" s="19" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="L88" s="19" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M88" s="19" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="N88" s="19" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O88" s="19" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="P88" s="19"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C89" s="17" t="n">
         <v>1</v>
@@ -8398,10 +8449,10 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B90" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C90" s="49" t="n">
         <f aca="false">Assumptions!$E$20*(1+Assumptions!$E$27)^(C$89-1)</f>
@@ -8455,10 +8506,10 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C91" s="48" t="n">
         <f aca="false">MIN(1,MAX(0,Assumptions!$E$21*(1+Assumptions!$E$28)^(C$89-1)))</f>
@@ -8512,10 +8563,10 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B92" s="14" t="s">
         <v>179</v>
-      </c>
-      <c r="B92" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="C92" s="45" t="n">
         <f aca="false">(1+Assumptions!$E$29)^(C$89-1)</f>
@@ -8572,7 +8623,7 @@
         <v>45</v>
       </c>
       <c r="B93" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C93" s="50" t="n">
         <f aca="false">Assumptions!$F$16*Assumptions!$F$15</f>
@@ -8632,7 +8683,7 @@
         <v>47</v>
       </c>
       <c r="B94" s="14" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C94" s="50" t="n">
         <f aca="false">C93*Assumptions!$E$19</f>
@@ -8689,10 +8740,10 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B95" s="14" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C95" s="50" t="n">
         <f aca="false">C94*Assumptions!$F$14</f>
@@ -8752,7 +8803,7 @@
         <v>51</v>
       </c>
       <c r="B96" s="14" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C96" s="50" t="n">
         <f aca="false">C95*C91</f>
@@ -8812,7 +8863,7 @@
         <v>53</v>
       </c>
       <c r="B97" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C97" s="53" t="n">
         <f aca="false">C96*C90</f>
@@ -8869,10 +8920,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="16" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B98" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C98" s="53" t="n">
         <f aca="false">C94*Assumptions!$E$22*C92</f>
@@ -8932,7 +8983,7 @@
         <v>57</v>
       </c>
       <c r="B99" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C99" s="53" t="n">
         <f aca="false">C96*Assumptions!$E$23*C92</f>
@@ -8989,10 +9040,10 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="B100" s="14" t="s">
         <v>198</v>
-      </c>
-      <c r="B100" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="C100" s="53" t="n">
         <f aca="false">C98+C99</f>
@@ -9052,7 +9103,7 @@
         <v>59</v>
       </c>
       <c r="B101" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C101" s="53" t="n">
         <f aca="false">C97-C100</f>
@@ -9109,10 +9160,10 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B102" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C102" s="53" t="n">
         <f aca="false">Assumptions!$E$24*C92</f>
@@ -9169,10 +9220,10 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B103" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C103" s="53" t="n">
         <f aca="false">C101-C102</f>
@@ -9229,10 +9280,10 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="16" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B104" s="14" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C104" s="53" t="n">
         <f aca="false">C95*(C90-Assumptions!$E$23*C92)</f>

</xml_diff>

<commit_message>
Add Sensitivity Analysis tab (fare x load factor contribution matrix)
Base-scenario, Month 1 matrix of contribution per completed flight across
nine fares and fifteen load factors, linked to Assumptions, with
loss/breakeven/profitable conditional formatting, flight-level vs
route-level breakeven load factors, three formula-driven insights and ten
validation checks that feed the Financial Model's overall status. Extend
audit_model.py to recompute the tab cell by cell, including settings
edge cases.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018QDw9YR2j2g8LL97XVTLTN
</commit_message>
<xml_diff>
--- a/Joby_Financial_Model.xlsx
+++ b/Joby_Financial_Model.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Financial Model" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Scenario Comparison" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Sensitivity Analysis" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" name="inp_capacity" vbProcedure="false">Assumptions!$F$14</definedName>
@@ -35,7 +36,7 @@
     <definedName function="false" hidden="false" name="out_fare" vbProcedure="false">'Financial Model'!$O$28</definedName>
     <definedName function="false" hidden="false" name="out_fixed" vbProcedure="false">'Financial Model'!$O$36</definedName>
     <definedName function="false" hidden="false" name="out_lf" vbProcedure="false">'Financial Model'!$O$17</definedName>
-    <definedName function="false" hidden="false" name="out_model_status" vbProcedure="false">'Financial Model'!$C$70</definedName>
+    <definedName function="false" hidden="false" name="out_model_status" vbProcedure="false">'Financial Model'!$C$71</definedName>
     <definedName function="false" hidden="false" name="out_pax" vbProcedure="false">'Financial Model'!$O$25</definedName>
     <definedName function="false" hidden="false" name="out_revenue" vbProcedure="false">'Financial Model'!$O$29</definedName>
     <definedName function="false" hidden="false" name="out_rop" vbProcedure="false">'Financial Model'!$O$37</definedName>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="372">
   <si>
     <t xml:space="preserve">Joby Aviation - Air Taxi Route Financial Model (Prototype)</t>
   </si>
@@ -113,10 +114,10 @@
     <t xml:space="preserve">Base / Upside / Downside computed side by side by an independent engine (rows 50+), with variance vs. Base.</t>
   </si>
   <si>
-    <t xml:space="preserve">Planned: Sensitivity Analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not yet built. Flex inputs via the inp_* defined names (or the Assumptions column F cells) and read results from the out_* defined names.</t>
+    <t xml:space="preserve">5. Sensitivity Analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base scenario, Month 1: contribution per completed flight across average fare (columns) x load factor (rows), shaded loss / breakeven / profitable. Flight-level vs. route-level breakeven load factor, three business insights and its own validation checks.</t>
   </si>
   <si>
     <t xml:space="preserve">Planned: Executive Dashboard</t>
@@ -845,6 +846,12 @@
     <t xml:space="preserve">Scenario Comparison (active case) matches Financial Model - passengers</t>
   </si>
   <si>
+    <t xml:space="preserve">Sensitivity Analysis checks pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status of the validation block on the Sensitivity Analysis tab.</t>
+  </si>
+  <si>
     <t xml:space="preserve">OVERALL MODEL STATUS</t>
   </si>
   <si>
@@ -966,6 +973,201 @@
   </si>
   <si>
     <t xml:space="preserve">Downside case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensitivity Analysis - Contribution per Completed Flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base scenario, Month 1 unit economics. Average fare (columns) x passenger load factor (rows). Linked to the Assumptions tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Base Scenario Inputs (Month 1, linked from Assumptions - edit there)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions, Route setup (all scenarios).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base average fare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions, Base column. Centre column of the matrix.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base passenger load factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions, Base column (Month 1, before demand growth).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct flight operating cost per completed flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions, Base column.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed route costs per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumptions, Base column. Used only for route-level breakeven.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed flights per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flights / month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating days x flights per day x Base completion rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Matrix Settings (editable, illustrative)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fare step between columns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columns run 4 steps below to 4 steps above the Base fare (floored at $0).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load factor - first row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top row of the matrix.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load factor step between rows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 rows; keep the last row at or below 100% (checked below).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breakeven band (+/-)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combinations within this band of $0 are shaded amber as 'breakeven'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative direct flight cost change</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used in insight 3 only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Breakeven Load Factor (Base, Month 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLIGHT-LEVEL breakeven load factor (contribution per flight = $0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula: Direct flight cost / (Seats x (Fare - Variable cost per passenger)). Covers flight-level variable costs only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed route costs per completed flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula: Monthly fixed route costs / completed flights per month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROUTE-LEVEL breakeven load factor (after fixed route costs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula: (Direct flight cost + Fixed route cost per flight) / (Seats x (Fare - Variable cost per passenger)). Route operating profit = $0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gap: route-level minus flight-level breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extra load factor needed to cover fixed route costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base load factor headroom vs. flight-level breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive = Base case covers its direct flight costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base load factor headroom vs. route-level breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive = Base case also covers fixed route costs (Month 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Contribution Profit per Completed Flight ($) - Average Fare (columns) x Load Factor (rows)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formula: Seats x LF x (Fare - Var. cost/pax) - Direct flight cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LF \ Fare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base case (Month 1):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(bold, boxed cell in the grid when on the axes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight-level breakeven LF at this fare</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route-level breakeven LF at this fare (after fixed costs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bold boxed cell = Base fare x Base load factor (when on the grid). Breakeven LF above 100% (red) cannot be reached at that fare.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legend (fare / load factor combinations)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loss-making (below -band)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breakeven (within +/- band)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profitable (above +band)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Business Insights (illustrative; text updates with the inputs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Sensitivity Validation Checks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Load factor axis within 0%-100%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix rises (or holds) with fare in every row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix rises with load factor wherever fare &gt; variable cost per passenger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base fare x Base LF cell = Base engine Month 1 contribution / flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight-level breakeven LF = Base engine Month 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route-level breakeven LF = Base engine Month 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contribution per flight at the flight-level breakeven LF = $0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route operating profit at the route-level breakeven LF = $0 (Month 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route-level breakeven &gt;= flight-level breakeven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legend counts sum to all 135 combinations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SENSITIVITY STATUS</t>
   </si>
 </sst>
 </file>
@@ -985,7 +1187,7 @@
     <numFmt numFmtId="173" formatCode="#,##0.0;\(#,##0.0\);\-"/>
     <numFmt numFmtId="174" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1093,8 +1295,16 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1129,6 +1339,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F7FC"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -1201,7 +1429,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="89">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1498,6 +1726,66 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="173" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1507,7 +1795,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill>
@@ -1535,6 +1823,47 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <u val="single"/>
+      </font>
+      <border diagonalUp="false" diagonalDown="false">
+        <left style="medium">
+          <color rgb="FF1F3864"/>
+        </left>
+        <right style="medium">
+          <color rgb="FF1F3864"/>
+        </right>
+        <top style="medium">
+          <color rgb="FF1F3864"/>
+        </top>
+        <bottom style="medium">
+          <color rgb="FF1F3864"/>
+        </bottom>
+        <diagonal/>
+      </border>
+    </dxf>
   </dxfs>
   <colors>
     <indexedColors>
@@ -1546,7 +1875,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF008000"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -1588,7 +1917,7 @@
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF006100"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
@@ -1814,8 +2143,8 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="str">
-        <f aca="false">'Financial Model'!$C$70</f>
-        <v>ALL 19 CHECKS PASS</v>
+        <f aca="false">'Financial Model'!$C$71</f>
+        <v>ALL 20 CHECKS PASS</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1900,7 +2229,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>20</v>
       </c>
@@ -2246,8 +2575,8 @@
         <v>87</v>
       </c>
       <c r="C7" s="6" t="str">
-        <f aca="false">'Financial Model'!$C$70</f>
-        <v>ALL 19 CHECKS PASS</v>
+        <f aca="false">'Financial Model'!$C$71</f>
+        <v>ALL 20 CHECKS PASS</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>88</v>
@@ -2824,7 +3153,7 @@
     <tabColor rgb="FF1F3864"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -5298,34 +5627,46 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="63" t="s">
+      <c r="A70" s="16" t="s">
         <v>264</v>
       </c>
-      <c r="B70" s="64"/>
-      <c r="C70" s="65" t="str">
-        <f aca="false">IF(COUNTIF($C$51:$C$69,"PASS")=19,"ALL 19 CHECKS PASS","REVIEW: "&amp;(19-COUNTIF($C$51:$C$69,"PASS"))&amp;" CHECK(S) FAILING")</f>
-        <v>ALL 19 CHECKS PASS</v>
-      </c>
-      <c r="D70" s="65"/>
-      <c r="E70" s="65"/>
-      <c r="F70" s="65"/>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="16" t="s">
+      <c r="C70" s="62" t="str">
+        <f aca="false">IF(LEFT('Sensitivity Analysis'!$B$71,3)="ALL","PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="D70" s="43" t="s">
         <v>265</v>
       </c>
-      <c r="C72" s="66" t="n">
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="63" t="s">
+        <v>266</v>
+      </c>
+      <c r="B71" s="64"/>
+      <c r="C71" s="65" t="str">
+        <f aca="false">IF(COUNTIF($C$51:$C$70,"PASS")=20,"ALL 20 CHECKS PASS","REVIEW: "&amp;(20-COUNTIF($C$51:$C$70,"PASS"))&amp;" CHECK(S) FAILING")</f>
+        <v>ALL 20 CHECKS PASS</v>
+      </c>
+      <c r="D71" s="65"/>
+      <c r="E71" s="65"/>
+      <c r="F71" s="65"/>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="16" t="s">
+        <v>267</v>
+      </c>
+      <c r="C73" s="66" t="n">
         <f aca="false">SUMPRODUCT((Assumptions!$F$21*$C$14:$N$14&gt;1)*1)</f>
         <v>0</v>
       </c>
-      <c r="D72" s="43" t="s">
-        <v>266</v>
+      <c r="D73" s="43" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A47:P47"/>
-    <mergeCell ref="C70:F70"/>
+    <mergeCell ref="C71:F71"/>
   </mergeCells>
   <conditionalFormatting sqref="C44:O44">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
@@ -5342,7 +5683,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C51:C69">
+  <conditionalFormatting sqref="C51:C70">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -5350,15 +5691,15 @@
       <formula>"FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C70">
+  <conditionalFormatting sqref="C71">
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>LEFT($C$70,3)="ALL"</formula>
+      <formula>LEFT($C$71,3)="ALL"</formula>
     </cfRule>
     <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>LEFT($C$70,3)&lt;&gt;"ALL"</formula>
+      <formula>LEFT($C$71,3)&lt;&gt;"ALL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C72">
+  <conditionalFormatting sqref="C73">
     <cfRule type="cellIs" priority="9" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5392,7 +5733,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5412,7 +5753,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5437,7 +5778,7 @@
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B5" s="19" t="s">
         <v>90</v>
@@ -5452,13 +5793,13 @@
         <v>92</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
@@ -5471,7 +5812,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
@@ -5494,7 +5835,7 @@
         <v>117</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C7" s="47" t="n">
         <f aca="false">Assumptions!$C$19</f>
@@ -5519,7 +5860,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>121</v>
@@ -5547,7 +5888,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>124</v>
@@ -5575,7 +5916,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>186</v>
@@ -5631,7 +5972,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>132</v>
@@ -5659,10 +6000,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C13" s="69" t="n">
         <f aca="false">Assumptions!$C$27</f>
@@ -5687,10 +6028,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C14" s="69" t="n">
         <f aca="false">Assumptions!$C$28</f>
@@ -5715,10 +6056,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
+        <v>284</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>282</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>280</v>
       </c>
       <c r="C15" s="69" t="n">
         <f aca="false">Assumptions!$C$29</f>
@@ -5743,7 +6084,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
@@ -5850,7 +6191,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>124</v>
@@ -5876,12 +6217,12 @@
         <v>-0.117519535379454</v>
       </c>
       <c r="H21" s="43" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>121</v>
@@ -5907,12 +6248,12 @@
         <v>-19.3738547164867</v>
       </c>
       <c r="H22" s="43" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>198</v>
@@ -5967,7 +6308,7 @@
         <v>118279.73668579</v>
       </c>
       <c r="H24" s="43" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5998,7 +6339,7 @@
         <v>-1560568.72150065</v>
       </c>
       <c r="H25" s="43" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6116,7 +6457,7 @@
         <v>-1714124.95879064</v>
       </c>
       <c r="H29" s="43" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6150,7 +6491,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>124</v>
@@ -6176,12 +6517,12 @@
         <v>0.126225158941928</v>
       </c>
       <c r="H31" s="43" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>124</v>
@@ -6207,15 +6548,15 @@
         <v>0.191282191636812</v>
       </c>
       <c r="H32" s="43" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="16" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C33" s="72" t="n">
         <f aca="false">COUNTIF(C67:N67,"&gt;0")</f>
@@ -6241,7 +6582,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -6327,7 +6668,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="59" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B40" s="59"/>
       <c r="C40" s="59"/>
@@ -6347,7 +6688,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="10"/>
@@ -6367,7 +6708,7 @@
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="18" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B52" s="19" t="s">
         <v>90</v>
@@ -7298,7 +7639,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="16" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B68" s="14" t="s">
         <v>198</v>
@@ -7358,7 +7699,7 @@
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="18" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B70" s="19" t="s">
         <v>90</v>
@@ -8289,7 +8630,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="16" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B86" s="14" t="s">
         <v>198</v>
@@ -8349,7 +8690,7 @@
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="18" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B88" s="19" t="s">
         <v>90</v>
@@ -9280,7 +9621,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="16" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B104" s="14" t="s">
         <v>198</v>
@@ -9378,4 +9719,1431 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FF1F3864"/>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:K71"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="3" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="41" t="n">
+        <f aca="false">Assumptions!$C$14</f>
+        <v>4</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D6" s="43" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="B7" s="67" t="n">
+        <f aca="false">Assumptions!$C$20</f>
+        <v>175</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="B8" s="47" t="n">
+        <f aca="false">Assumptions!$C$21</f>
+        <v>0.6</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="43" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="B9" s="67" t="n">
+        <f aca="false">Assumptions!$C$22</f>
+        <v>300</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="67" t="n">
+        <f aca="false">Assumptions!$C$23</f>
+        <v>12</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="43" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="B11" s="68" t="n">
+        <f aca="false">Assumptions!$C$24</f>
+        <v>90000</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" s="43" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="B12" s="74" t="n">
+        <f aca="false">Assumptions!$C$16*Assumptions!$C$15*Assumptions!$C$19</f>
+        <v>851.2</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="D12" s="43" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="B15" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D15" s="43" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
+        <v>325</v>
+      </c>
+      <c r="B16" s="28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D16" s="43" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
+        <v>327</v>
+      </c>
+      <c r="B17" s="28" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D17" s="43" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>331</v>
+      </c>
+      <c r="B19" s="30" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D19" s="43" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="B22" s="75" t="n">
+        <f aca="false">IF($B$7&gt;$B$10,$B$9/($B$6*($B$7-$B$10)),"n.m.")</f>
+        <v>0.460122699386503</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="16" t="s">
+        <v>336</v>
+      </c>
+      <c r="B23" s="49" t="n">
+        <f aca="false">IF($B$12&gt;0,$B$11/$B$12,"n.m.")</f>
+        <v>105.733082706767</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="B24" s="75" t="n">
+        <f aca="false">IF(AND($B$7&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*($B$7-$B$10)),"n.m.")</f>
+        <v>0.622290004151483</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D24" s="43" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16" t="s">
+        <v>340</v>
+      </c>
+      <c r="B25" s="75" t="n">
+        <f aca="false">IF(AND(ISNUMBER($B$24),ISNUMBER($B$22)),$B$24-$B$22,"n.m.")</f>
+        <v>0.16216730476498</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D25" s="43" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="B26" s="75" t="n">
+        <f aca="false">IF(ISNUMBER($B$22),$B$8-$B$22,"n.m.")</f>
+        <v>0.139877300613497</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D26" s="43" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>344</v>
+      </c>
+      <c r="B27" s="75" t="n">
+        <f aca="false">IF(ISNUMBER($B$24),$B$8-$B$24,"n.m.")</f>
+        <v>-0.0222900041514831</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D27" s="43" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="76" t="s">
+        <v>347</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>348</v>
+      </c>
+      <c r="C30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND($B$7-4*$B$15,2))</f>
+        <v>115</v>
+      </c>
+      <c r="D30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(C30+$B$15,2))</f>
+        <v>130</v>
+      </c>
+      <c r="E30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(D30+$B$15,2))</f>
+        <v>145</v>
+      </c>
+      <c r="F30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(E30+$B$15,2))</f>
+        <v>160</v>
+      </c>
+      <c r="G30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(F30+$B$15,2))</f>
+        <v>175</v>
+      </c>
+      <c r="H30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(G30+$B$15,2))</f>
+        <v>190</v>
+      </c>
+      <c r="I30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(H30+$B$15,2))</f>
+        <v>205</v>
+      </c>
+      <c r="J30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(I30+$B$15,2))</f>
+        <v>220</v>
+      </c>
+      <c r="K30" s="77" t="n">
+        <f aca="false">MAX(0,ROUND(J30+$B$15,2))</f>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="78" t="s">
+        <v>349</v>
+      </c>
+      <c r="B31" s="79" t="n">
+        <f aca="false">ROUND($B$16,4)</f>
+        <v>0.3</v>
+      </c>
+      <c r="C31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(C$30-$B$10)-$B$9</f>
+        <v>-176.4</v>
+      </c>
+      <c r="D31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(D$30-$B$10)-$B$9</f>
+        <v>-158.4</v>
+      </c>
+      <c r="E31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(E$30-$B$10)-$B$9</f>
+        <v>-140.4</v>
+      </c>
+      <c r="F31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(F$30-$B$10)-$B$9</f>
+        <v>-122.4</v>
+      </c>
+      <c r="G31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(G$30-$B$10)-$B$9</f>
+        <v>-104.4</v>
+      </c>
+      <c r="H31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(H$30-$B$10)-$B$9</f>
+        <v>-86.4</v>
+      </c>
+      <c r="I31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(I$30-$B$10)-$B$9</f>
+        <v>-68.4</v>
+      </c>
+      <c r="J31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(J$30-$B$10)-$B$9</f>
+        <v>-50.4</v>
+      </c>
+      <c r="K31" s="80" t="n">
+        <f aca="false">$B$6*$B31*(K$30-$B$10)-$B$9</f>
+        <v>-32.4</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="81" t="str">
+        <f aca="false">TEXT($B$7,"$0.00")&amp;" fare x "&amp;TEXT($B$8,"0.0%")&amp;" load factor = "&amp;TEXT($B$6*$B$8*($B$7-$B$10)-$B$9,"$#,##0.00")&amp;" per completed flight"</f>
+        <v>$175.00 fare x 60.0% load factor = $91.20 per completed flight</v>
+      </c>
+      <c r="B32" s="79" t="n">
+        <f aca="false">ROUND(B31+$B$17,4)</f>
+        <v>0.35</v>
+      </c>
+      <c r="C32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(C$30-$B$10)-$B$9</f>
+        <v>-155.8</v>
+      </c>
+      <c r="D32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(D$30-$B$10)-$B$9</f>
+        <v>-134.8</v>
+      </c>
+      <c r="E32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(E$30-$B$10)-$B$9</f>
+        <v>-113.8</v>
+      </c>
+      <c r="F32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(F$30-$B$10)-$B$9</f>
+        <v>-92.8</v>
+      </c>
+      <c r="G32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(G$30-$B$10)-$B$9</f>
+        <v>-71.8</v>
+      </c>
+      <c r="H32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(H$30-$B$10)-$B$9</f>
+        <v>-50.8</v>
+      </c>
+      <c r="I32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(I$30-$B$10)-$B$9</f>
+        <v>-29.8</v>
+      </c>
+      <c r="J32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(J$30-$B$10)-$B$9</f>
+        <v>-8.80000000000001</v>
+      </c>
+      <c r="K32" s="80" t="n">
+        <f aca="false">$B$6*$B32*(K$30-$B$10)-$B$9</f>
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="82" t="s">
+        <v>350</v>
+      </c>
+      <c r="B33" s="79" t="n">
+        <f aca="false">ROUND(B32+$B$17,4)</f>
+        <v>0.4</v>
+      </c>
+      <c r="C33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(C$30-$B$10)-$B$9</f>
+        <v>-135.2</v>
+      </c>
+      <c r="D33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(D$30-$B$10)-$B$9</f>
+        <v>-111.2</v>
+      </c>
+      <c r="E33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(E$30-$B$10)-$B$9</f>
+        <v>-87.2</v>
+      </c>
+      <c r="F33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(F$30-$B$10)-$B$9</f>
+        <v>-63.2</v>
+      </c>
+      <c r="G33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(G$30-$B$10)-$B$9</f>
+        <v>-39.2</v>
+      </c>
+      <c r="H33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(H$30-$B$10)-$B$9</f>
+        <v>-15.2</v>
+      </c>
+      <c r="I33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(I$30-$B$10)-$B$9</f>
+        <v>8.80000000000001</v>
+      </c>
+      <c r="J33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(J$30-$B$10)-$B$9</f>
+        <v>32.8</v>
+      </c>
+      <c r="K33" s="80" t="n">
+        <f aca="false">$B$6*$B33*(K$30-$B$10)-$B$9</f>
+        <v>56.8</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="79" t="n">
+        <f aca="false">ROUND(B33+$B$17,4)</f>
+        <v>0.45</v>
+      </c>
+      <c r="C34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(C$30-$B$10)-$B$9</f>
+        <v>-114.6</v>
+      </c>
+      <c r="D34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(D$30-$B$10)-$B$9</f>
+        <v>-87.6</v>
+      </c>
+      <c r="E34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(E$30-$B$10)-$B$9</f>
+        <v>-60.6</v>
+      </c>
+      <c r="F34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(F$30-$B$10)-$B$9</f>
+        <v>-33.6</v>
+      </c>
+      <c r="G34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(G$30-$B$10)-$B$9</f>
+        <v>-6.59999999999997</v>
+      </c>
+      <c r="H34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(H$30-$B$10)-$B$9</f>
+        <v>20.4</v>
+      </c>
+      <c r="I34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(I$30-$B$10)-$B$9</f>
+        <v>47.4</v>
+      </c>
+      <c r="J34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(J$30-$B$10)-$B$9</f>
+        <v>74.4</v>
+      </c>
+      <c r="K34" s="80" t="n">
+        <f aca="false">$B$6*$B34*(K$30-$B$10)-$B$9</f>
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="79" t="n">
+        <f aca="false">ROUND(B34+$B$17,4)</f>
+        <v>0.5</v>
+      </c>
+      <c r="C35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(C$30-$B$10)-$B$9</f>
+        <v>-94</v>
+      </c>
+      <c r="D35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(D$30-$B$10)-$B$9</f>
+        <v>-64</v>
+      </c>
+      <c r="E35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(E$30-$B$10)-$B$9</f>
+        <v>-34</v>
+      </c>
+      <c r="F35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(F$30-$B$10)-$B$9</f>
+        <v>-4</v>
+      </c>
+      <c r="G35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(G$30-$B$10)-$B$9</f>
+        <v>26</v>
+      </c>
+      <c r="H35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(H$30-$B$10)-$B$9</f>
+        <v>56</v>
+      </c>
+      <c r="I35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(I$30-$B$10)-$B$9</f>
+        <v>86</v>
+      </c>
+      <c r="J35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(J$30-$B$10)-$B$9</f>
+        <v>116</v>
+      </c>
+      <c r="K35" s="80" t="n">
+        <f aca="false">$B$6*$B35*(K$30-$B$10)-$B$9</f>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="79" t="n">
+        <f aca="false">ROUND(B35+$B$17,4)</f>
+        <v>0.55</v>
+      </c>
+      <c r="C36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(C$30-$B$10)-$B$9</f>
+        <v>-73.4</v>
+      </c>
+      <c r="D36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(D$30-$B$10)-$B$9</f>
+        <v>-40.4</v>
+      </c>
+      <c r="E36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(E$30-$B$10)-$B$9</f>
+        <v>-7.39999999999998</v>
+      </c>
+      <c r="F36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(F$30-$B$10)-$B$9</f>
+        <v>25.6</v>
+      </c>
+      <c r="G36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(G$30-$B$10)-$B$9</f>
+        <v>58.6</v>
+      </c>
+      <c r="H36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(H$30-$B$10)-$B$9</f>
+        <v>91.6</v>
+      </c>
+      <c r="I36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(I$30-$B$10)-$B$9</f>
+        <v>124.6</v>
+      </c>
+      <c r="J36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(J$30-$B$10)-$B$9</f>
+        <v>157.6</v>
+      </c>
+      <c r="K36" s="80" t="n">
+        <f aca="false">$B$6*$B36*(K$30-$B$10)-$B$9</f>
+        <v>190.6</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="79" t="n">
+        <f aca="false">ROUND(B36+$B$17,4)</f>
+        <v>0.6</v>
+      </c>
+      <c r="C37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(C$30-$B$10)-$B$9</f>
+        <v>-52.8</v>
+      </c>
+      <c r="D37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(D$30-$B$10)-$B$9</f>
+        <v>-16.8</v>
+      </c>
+      <c r="E37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(E$30-$B$10)-$B$9</f>
+        <v>19.2</v>
+      </c>
+      <c r="F37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(F$30-$B$10)-$B$9</f>
+        <v>55.2</v>
+      </c>
+      <c r="G37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(G$30-$B$10)-$B$9</f>
+        <v>91.2</v>
+      </c>
+      <c r="H37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(H$30-$B$10)-$B$9</f>
+        <v>127.2</v>
+      </c>
+      <c r="I37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(I$30-$B$10)-$B$9</f>
+        <v>163.2</v>
+      </c>
+      <c r="J37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(J$30-$B$10)-$B$9</f>
+        <v>199.2</v>
+      </c>
+      <c r="K37" s="80" t="n">
+        <f aca="false">$B$6*$B37*(K$30-$B$10)-$B$9</f>
+        <v>235.2</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="79" t="n">
+        <f aca="false">ROUND(B37+$B$17,4)</f>
+        <v>0.65</v>
+      </c>
+      <c r="C38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(C$30-$B$10)-$B$9</f>
+        <v>-32.2</v>
+      </c>
+      <c r="D38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(D$30-$B$10)-$B$9</f>
+        <v>6.80000000000001</v>
+      </c>
+      <c r="E38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(E$30-$B$10)-$B$9</f>
+        <v>45.8</v>
+      </c>
+      <c r="F38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(F$30-$B$10)-$B$9</f>
+        <v>84.8</v>
+      </c>
+      <c r="G38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(G$30-$B$10)-$B$9</f>
+        <v>123.8</v>
+      </c>
+      <c r="H38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(H$30-$B$10)-$B$9</f>
+        <v>162.8</v>
+      </c>
+      <c r="I38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(I$30-$B$10)-$B$9</f>
+        <v>201.8</v>
+      </c>
+      <c r="J38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(J$30-$B$10)-$B$9</f>
+        <v>240.8</v>
+      </c>
+      <c r="K38" s="80" t="n">
+        <f aca="false">$B$6*$B38*(K$30-$B$10)-$B$9</f>
+        <v>279.8</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B39" s="79" t="n">
+        <f aca="false">ROUND(B38+$B$17,4)</f>
+        <v>0.7</v>
+      </c>
+      <c r="C39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(C$30-$B$10)-$B$9</f>
+        <v>-11.6</v>
+      </c>
+      <c r="D39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(D$30-$B$10)-$B$9</f>
+        <v>30.4</v>
+      </c>
+      <c r="E39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(E$30-$B$10)-$B$9</f>
+        <v>72.4</v>
+      </c>
+      <c r="F39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(F$30-$B$10)-$B$9</f>
+        <v>114.4</v>
+      </c>
+      <c r="G39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(G$30-$B$10)-$B$9</f>
+        <v>156.4</v>
+      </c>
+      <c r="H39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(H$30-$B$10)-$B$9</f>
+        <v>198.4</v>
+      </c>
+      <c r="I39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(I$30-$B$10)-$B$9</f>
+        <v>240.4</v>
+      </c>
+      <c r="J39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(J$30-$B$10)-$B$9</f>
+        <v>282.4</v>
+      </c>
+      <c r="K39" s="80" t="n">
+        <f aca="false">$B$6*$B39*(K$30-$B$10)-$B$9</f>
+        <v>324.4</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B40" s="79" t="n">
+        <f aca="false">ROUND(B39+$B$17,4)</f>
+        <v>0.75</v>
+      </c>
+      <c r="C40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(C$30-$B$10)-$B$9</f>
+        <v>9</v>
+      </c>
+      <c r="D40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(D$30-$B$10)-$B$9</f>
+        <v>54</v>
+      </c>
+      <c r="E40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(E$30-$B$10)-$B$9</f>
+        <v>99</v>
+      </c>
+      <c r="F40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(F$30-$B$10)-$B$9</f>
+        <v>144</v>
+      </c>
+      <c r="G40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(G$30-$B$10)-$B$9</f>
+        <v>189</v>
+      </c>
+      <c r="H40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(H$30-$B$10)-$B$9</f>
+        <v>234</v>
+      </c>
+      <c r="I40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(I$30-$B$10)-$B$9</f>
+        <v>279</v>
+      </c>
+      <c r="J40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(J$30-$B$10)-$B$9</f>
+        <v>324</v>
+      </c>
+      <c r="K40" s="80" t="n">
+        <f aca="false">$B$6*$B40*(K$30-$B$10)-$B$9</f>
+        <v>369</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B41" s="79" t="n">
+        <f aca="false">ROUND(B40+$B$17,4)</f>
+        <v>0.8</v>
+      </c>
+      <c r="C41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(C$30-$B$10)-$B$9</f>
+        <v>29.6</v>
+      </c>
+      <c r="D41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(D$30-$B$10)-$B$9</f>
+        <v>77.6</v>
+      </c>
+      <c r="E41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(E$30-$B$10)-$B$9</f>
+        <v>125.6</v>
+      </c>
+      <c r="F41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(F$30-$B$10)-$B$9</f>
+        <v>173.6</v>
+      </c>
+      <c r="G41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(G$30-$B$10)-$B$9</f>
+        <v>221.6</v>
+      </c>
+      <c r="H41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(H$30-$B$10)-$B$9</f>
+        <v>269.6</v>
+      </c>
+      <c r="I41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(I$30-$B$10)-$B$9</f>
+        <v>317.6</v>
+      </c>
+      <c r="J41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(J$30-$B$10)-$B$9</f>
+        <v>365.6</v>
+      </c>
+      <c r="K41" s="80" t="n">
+        <f aca="false">$B$6*$B41*(K$30-$B$10)-$B$9</f>
+        <v>413.6</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B42" s="79" t="n">
+        <f aca="false">ROUND(B41+$B$17,4)</f>
+        <v>0.85</v>
+      </c>
+      <c r="C42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(C$30-$B$10)-$B$9</f>
+        <v>50.2</v>
+      </c>
+      <c r="D42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(D$30-$B$10)-$B$9</f>
+        <v>101.2</v>
+      </c>
+      <c r="E42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(E$30-$B$10)-$B$9</f>
+        <v>152.2</v>
+      </c>
+      <c r="F42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(F$30-$B$10)-$B$9</f>
+        <v>203.2</v>
+      </c>
+      <c r="G42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(G$30-$B$10)-$B$9</f>
+        <v>254.2</v>
+      </c>
+      <c r="H42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(H$30-$B$10)-$B$9</f>
+        <v>305.2</v>
+      </c>
+      <c r="I42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(I$30-$B$10)-$B$9</f>
+        <v>356.2</v>
+      </c>
+      <c r="J42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(J$30-$B$10)-$B$9</f>
+        <v>407.2</v>
+      </c>
+      <c r="K42" s="80" t="n">
+        <f aca="false">$B$6*$B42*(K$30-$B$10)-$B$9</f>
+        <v>458.2</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B43" s="79" t="n">
+        <f aca="false">ROUND(B42+$B$17,4)</f>
+        <v>0.9</v>
+      </c>
+      <c r="C43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(C$30-$B$10)-$B$9</f>
+        <v>70.8</v>
+      </c>
+      <c r="D43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(D$30-$B$10)-$B$9</f>
+        <v>124.8</v>
+      </c>
+      <c r="E43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(E$30-$B$10)-$B$9</f>
+        <v>178.8</v>
+      </c>
+      <c r="F43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(F$30-$B$10)-$B$9</f>
+        <v>232.8</v>
+      </c>
+      <c r="G43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(G$30-$B$10)-$B$9</f>
+        <v>286.8</v>
+      </c>
+      <c r="H43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(H$30-$B$10)-$B$9</f>
+        <v>340.8</v>
+      </c>
+      <c r="I43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(I$30-$B$10)-$B$9</f>
+        <v>394.8</v>
+      </c>
+      <c r="J43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(J$30-$B$10)-$B$9</f>
+        <v>448.8</v>
+      </c>
+      <c r="K43" s="80" t="n">
+        <f aca="false">$B$6*$B43*(K$30-$B$10)-$B$9</f>
+        <v>502.8</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="79" t="n">
+        <f aca="false">ROUND(B43+$B$17,4)</f>
+        <v>0.95</v>
+      </c>
+      <c r="C44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(C$30-$B$10)-$B$9</f>
+        <v>91.4</v>
+      </c>
+      <c r="D44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(D$30-$B$10)-$B$9</f>
+        <v>148.4</v>
+      </c>
+      <c r="E44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(E$30-$B$10)-$B$9</f>
+        <v>205.4</v>
+      </c>
+      <c r="F44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(F$30-$B$10)-$B$9</f>
+        <v>262.4</v>
+      </c>
+      <c r="G44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(G$30-$B$10)-$B$9</f>
+        <v>319.4</v>
+      </c>
+      <c r="H44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(H$30-$B$10)-$B$9</f>
+        <v>376.4</v>
+      </c>
+      <c r="I44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(I$30-$B$10)-$B$9</f>
+        <v>433.4</v>
+      </c>
+      <c r="J44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(J$30-$B$10)-$B$9</f>
+        <v>490.4</v>
+      </c>
+      <c r="K44" s="80" t="n">
+        <f aca="false">$B$6*$B44*(K$30-$B$10)-$B$9</f>
+        <v>547.4</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="79" t="n">
+        <f aca="false">ROUND(B44+$B$17,4)</f>
+        <v>1</v>
+      </c>
+      <c r="C45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(C$30-$B$10)-$B$9</f>
+        <v>112</v>
+      </c>
+      <c r="D45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(D$30-$B$10)-$B$9</f>
+        <v>172</v>
+      </c>
+      <c r="E45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(E$30-$B$10)-$B$9</f>
+        <v>232</v>
+      </c>
+      <c r="F45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(F$30-$B$10)-$B$9</f>
+        <v>292</v>
+      </c>
+      <c r="G45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(G$30-$B$10)-$B$9</f>
+        <v>352</v>
+      </c>
+      <c r="H45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(H$30-$B$10)-$B$9</f>
+        <v>412</v>
+      </c>
+      <c r="I45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(I$30-$B$10)-$B$9</f>
+        <v>472</v>
+      </c>
+      <c r="J45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(J$30-$B$10)-$B$9</f>
+        <v>532</v>
+      </c>
+      <c r="K45" s="80" t="n">
+        <f aca="false">$B$6*$B45*(K$30-$B$10)-$B$9</f>
+        <v>592</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="83" t="s">
+        <v>351</v>
+      </c>
+      <c r="B46" s="83"/>
+      <c r="C46" s="84" t="n">
+        <f aca="false">IF(C$30&gt;$B$10,($B$9)/($B$6*(C$30-$B$10)),"n.m.")</f>
+        <v>0.728155339805825</v>
+      </c>
+      <c r="D46" s="84" t="n">
+        <f aca="false">IF(D$30&gt;$B$10,($B$9)/($B$6*(D$30-$B$10)),"n.m.")</f>
+        <v>0.635593220338983</v>
+      </c>
+      <c r="E46" s="84" t="n">
+        <f aca="false">IF(E$30&gt;$B$10,($B$9)/($B$6*(E$30-$B$10)),"n.m.")</f>
+        <v>0.56390977443609</v>
+      </c>
+      <c r="F46" s="84" t="n">
+        <f aca="false">IF(F$30&gt;$B$10,($B$9)/($B$6*(F$30-$B$10)),"n.m.")</f>
+        <v>0.506756756756757</v>
+      </c>
+      <c r="G46" s="84" t="n">
+        <f aca="false">IF(G$30&gt;$B$10,($B$9)/($B$6*(G$30-$B$10)),"n.m.")</f>
+        <v>0.460122699386503</v>
+      </c>
+      <c r="H46" s="84" t="n">
+        <f aca="false">IF(H$30&gt;$B$10,($B$9)/($B$6*(H$30-$B$10)),"n.m.")</f>
+        <v>0.421348314606742</v>
+      </c>
+      <c r="I46" s="84" t="n">
+        <f aca="false">IF(I$30&gt;$B$10,($B$9)/($B$6*(I$30-$B$10)),"n.m.")</f>
+        <v>0.38860103626943</v>
+      </c>
+      <c r="J46" s="84" t="n">
+        <f aca="false">IF(J$30&gt;$B$10,($B$9)/($B$6*(J$30-$B$10)),"n.m.")</f>
+        <v>0.360576923076923</v>
+      </c>
+      <c r="K46" s="84" t="n">
+        <f aca="false">IF(K$30&gt;$B$10,($B$9)/($B$6*(K$30-$B$10)),"n.m.")</f>
+        <v>0.336322869955157</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="83" t="s">
+        <v>352</v>
+      </c>
+      <c r="B47" s="83"/>
+      <c r="C47" s="84" t="n">
+        <f aca="false">IF(AND(C$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(C$30-$B$10)),"n.m.")</f>
+        <v>0.984789035696036</v>
+      </c>
+      <c r="D47" s="84" t="n">
+        <f aca="false">IF(AND(D$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(D$30-$B$10)),"n.m.")</f>
+        <v>0.859603988785523</v>
+      </c>
+      <c r="E47" s="84" t="n">
+        <f aca="false">IF(AND(E$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(E$30-$B$10)),"n.m.")</f>
+        <v>0.762656170501442</v>
+      </c>
+      <c r="F47" s="84" t="n">
+        <f aca="false">IF(AND(F$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(F$30-$B$10)),"n.m.")</f>
+        <v>0.685359937004674</v>
+      </c>
+      <c r="G47" s="84" t="n">
+        <f aca="false">IF(AND(G$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(G$30-$B$10)),"n.m.")</f>
+        <v>0.622290004151483</v>
+      </c>
+      <c r="H47" s="84" t="n">
+        <f aca="false">IF(AND(H$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(H$30-$B$10)),"n.m.")</f>
+        <v>0.569849835262313</v>
+      </c>
+      <c r="I47" s="84" t="n">
+        <f aca="false">IF(AND(I$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(I$30-$B$10)),"n.m.")</f>
+        <v>0.525560987962133</v>
+      </c>
+      <c r="J47" s="84" t="n">
+        <f aca="false">IF(AND(J$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(J$30-$B$10)),"n.m.")</f>
+        <v>0.487659955176403</v>
+      </c>
+      <c r="K47" s="84" t="n">
+        <f aca="false">IF(AND(K$30&gt;$B$10,ISNUMBER($B$23)),($B$9+$B$23)/($B$6*(K$30-$B$10)),"n.m.")</f>
+        <v>0.454857716038976</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="B50" s="62" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="85" t="s">
+        <v>356</v>
+      </c>
+      <c r="B51" s="17" t="n">
+        <f aca="false">COUNTIF($C$31:$K$45,"&lt;"&amp;-$B$18)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="86" t="s">
+        <v>357</v>
+      </c>
+      <c r="B52" s="17" t="n">
+        <f aca="false">COUNTIFS($C$31:$K$45,"&gt;="&amp;-$B$18,$C$31:$K$45,"&lt;="&amp;$B$18)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="87" t="s">
+        <v>358</v>
+      </c>
+      <c r="B53" s="17" t="n">
+        <f aca="false">COUNTIF($C$31:$K$45,"&gt;"&amp;$B$18)</f>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="B55" s="10"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10"/>
+    </row>
+    <row r="56" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="36" t="str">
+        <f aca="false">IFERROR("1. Pricing: at the Base "&amp;TEXT($B$8,"0%")&amp;" load factor, every "&amp;TEXT($B$15,"$0")&amp;" change in average fare moves contribution per completed flight by "&amp;TEXT($B$6*$B$8*$B$15,"$#,##0")&amp;". Across the matrix the flight-level breakeven load factor falls from "&amp;TEXT($C$46,"0.0%")&amp;" at "&amp;TEXT($C$30,"$0")&amp;" to "&amp;TEXT($K$46,"0.0%")&amp;" at "&amp;TEXT($K$30,"$0")&amp;", so pricing power directly widens the margin of safety against weak demand.","Insight not meaningful: Base fare does not exceed the variable cost per passenger, or there are no completed flights.")</f>
+        <v>1. Pricing: at the Base 60% load factor, every $15 change in average fare moves contribution per completed flight by $36. Across the matrix the flight-level breakeven load factor falls from 72.8% at $115 to 33.6% at $235, so pricing power directly widens the margin of safety against weak demand.</v>
+      </c>
+      <c r="B56" s="36"/>
+      <c r="C56" s="36"/>
+      <c r="D56" s="36"/>
+      <c r="E56" s="36"/>
+      <c r="F56" s="36"/>
+      <c r="G56" s="36"/>
+      <c r="H56" s="36"/>
+      <c r="I56" s="36"/>
+      <c r="J56" s="36"/>
+      <c r="K56" s="36"/>
+    </row>
+    <row r="57" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="36" t="str">
+        <f aca="false">IFERROR("2. Demand: each "&amp;TEXT($B$17*100,"0")&amp;"-point change in load factor moves contribution per flight by "&amp;TEXT($B$6*$B$17*($B$7-$B$10),"$#,##0")&amp;". The Base route covers its direct flight costs above a "&amp;TEXT($B$22,"0.0%")&amp;" load factor but needs "&amp;TEXT($B$24,"0.0%")&amp;" to also cover fixed route costs - a "&amp;TEXT($B$25*100,"0.0")&amp;"-point gap that only more completed flights, a higher fare or lower fixed costs can close.","Insight not meaningful: Base fare does not exceed the variable cost per passenger, or there are no completed flights.")</f>
+        <v>2. Demand: each 5-point change in load factor moves contribution per flight by $33. The Base route covers its direct flight costs above a 46.0% load factor but needs 62.2% to also cover fixed route costs - a 16.2-point gap that only more completed flights, a higher fare or lower fixed costs can close.</v>
+      </c>
+      <c r="B57" s="36"/>
+      <c r="C57" s="36"/>
+      <c r="D57" s="36"/>
+      <c r="E57" s="36"/>
+      <c r="F57" s="36"/>
+      <c r="G57" s="36"/>
+      <c r="H57" s="36"/>
+      <c r="I57" s="36"/>
+      <c r="J57" s="36"/>
+      <c r="K57" s="36"/>
+    </row>
+    <row r="58" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="36" t="str">
+        <f aca="false">IFERROR("3. Cost: a "&amp;TEXT($B$19,"$0")&amp;" increase in direct flight cost per completed flight cuts contribution per flight by the same "&amp;TEXT($B$19,"$0")&amp;" at every fare and load factor and raises the flight-level breakeven load factor by "&amp;TEXT($B$19/($B$6*($B$7-$B$10))*100,"0.0")&amp;" points. Per-passenger costs instead reduce the net fare earned on every seat sold, so they matter most when load factors are high.","Insight not meaningful: Base fare does not exceed the variable cost per passenger, or there are no completed flights.")</f>
+        <v>3. Cost: a $25 increase in direct flight cost per completed flight cuts contribution per flight by the same $25 at every fare and load factor and raises the flight-level breakeven load factor by 3.8 points. Per-passenger costs instead reduce the net fare earned on every seat sold, so they matter most when load factors are high.</v>
+      </c>
+      <c r="B58" s="36"/>
+      <c r="C58" s="36"/>
+      <c r="D58" s="36"/>
+      <c r="E58" s="36"/>
+      <c r="F58" s="36"/>
+      <c r="G58" s="36"/>
+      <c r="H58" s="36"/>
+      <c r="I58" s="36"/>
+      <c r="J58" s="36"/>
+      <c r="K58" s="36"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10"/>
+      <c r="I60" s="10"/>
+      <c r="J60" s="10"/>
+      <c r="K60" s="10"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="16" t="s">
+        <v>361</v>
+      </c>
+      <c r="B61" s="62" t="str">
+        <f aca="false">IF(AND(MIN($B$31:$B$45)&gt;=0,MAX($B$31:$B$45)&lt;=1),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="16" t="s">
+        <v>362</v>
+      </c>
+      <c r="B62" s="62" t="str">
+        <f aca="false">IF(SUMPRODUCT(($D$31:$K$45&lt;$C$31:$J$45-0.000001)*1)=0,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="16" t="s">
+        <v>363</v>
+      </c>
+      <c r="B63" s="62" t="str">
+        <f aca="false">IF(SUMPRODUCT(($C$32:$K$45&lt;$C$31:$K$44-0.000001)*($C$30:$K$30&gt;$B$10))=0,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="B64" s="62" t="str">
+        <f aca="false">IF(OR('Scenario Comparison'!$C$58=0,SUMPRODUCT(($B$31:$B$45=$B$8)*($C$30:$K$30=$B$7))&lt;&gt;1),"N/A",IF(ABS(SUMPRODUCT(($B$31:$B$45=$B$8)*($C$30:$K$30=$B$7)*$C$31:$K$45)-'Scenario Comparison'!$C$65/'Scenario Comparison'!$C$58)&lt;0.01,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="16" t="s">
+        <v>365</v>
+      </c>
+      <c r="B65" s="62" t="str">
+        <f aca="false">IF(OR(NOT(ISNUMBER($B$22)),'Scenario Comparison'!$C$68&lt;=0),"N/A",IF(ABS($B$22-'Scenario Comparison'!$C$62/'Scenario Comparison'!$C$68)&lt;0.000001,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="16" t="s">
+        <v>366</v>
+      </c>
+      <c r="B66" s="62" t="str">
+        <f aca="false">IF(OR(NOT(ISNUMBER($B$24)),'Scenario Comparison'!$C$68&lt;=0),"N/A",IF(ABS($B$24-('Scenario Comparison'!$C$62+'Scenario Comparison'!$C$66)/'Scenario Comparison'!$C$68)&lt;0.000001,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="16" t="s">
+        <v>367</v>
+      </c>
+      <c r="B67" s="62" t="str">
+        <f aca="false">IF(NOT(ISNUMBER($B$22)),"N/A",IF(ABS($B$6*$B$22*($B$7-$B$10)-$B$9)&lt;0.01,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="16" t="s">
+        <v>368</v>
+      </c>
+      <c r="B68" s="62" t="str">
+        <f aca="false">IF(NOT(ISNUMBER($B$24)),"N/A",IF(ABS($B$12*($B$6*$B$24*($B$7-$B$10)-$B$9)-$B$11)&lt;0.01,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="16" t="s">
+        <v>369</v>
+      </c>
+      <c r="B69" s="62" t="str">
+        <f aca="false">IF(NOT(ISNUMBER($B$25)),"N/A",IF($B$25&gt;=-0.000001,"PASS","FAIL"))</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="16" t="s">
+        <v>370</v>
+      </c>
+      <c r="B70" s="62" t="str">
+        <f aca="false">IF(SUM($B$51:$B$53)=135,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="B71" s="88" t="str">
+        <f aca="false">IF(COUNTIF($B$61:$B$70,"FAIL")=0,"ALL SENSITIVITY CHECKS PASS ("&amp;COUNTIF($B$61:$B$70,"PASS")&amp;" pass, "&amp;COUNTIF($B$61:$B$70,"N/A")&amp;" n/a)","REVIEW: "&amp;COUNTIF($B$61:$B$70,"FAIL")&amp;" FAILING")</f>
+        <v>ALL SENSITIVITY CHECKS PASS (10 pass, 0 n/a)</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A56:K56"/>
+    <mergeCell ref="A57:K57"/>
+    <mergeCell ref="A58:K58"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C31:K45">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>ABS(C31)&lt;=$B$18</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>C31&lt;-$B$18</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>C31&gt;$B$18</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>AND(C$30=$B$7,$B31=$B$8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C46:K46">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>AND(ISNUMBER(C46),C46&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C47:K47">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>AND(ISNUMBER(C47),C47&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B61:B70">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B71">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>LEFT($B$71,3)="ALL"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>LEFT($B$71,3)&lt;&gt;"ALL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" error="Enter a rate between 0% and 100%." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B16:B17" type="decimal">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Enter a value of zero or more." errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B15 B18:B19" type="decimal">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>